<commit_message>
Take weekly tiffin orders on the website
The Order page gets its own order form, built from menu.json: a combo,
exactly as many curries as it includes, roti add-ons, specials and a
delivery zone, with a running total and free delivery over the set
amount. Orders post to a Google Apps Script (scripts/order-sheet.gs)
that re-prices them from the live menu, adds a row to an Orders sheet
and emails Chaitrali and the customer.

The form switches on once Business Info's new Order Sheet Link holds the
script's web-app URL; until then every Order button keeps opening the
Google Form. README covers the one-time setup.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ChaitralisKitchen_ContentPack.xlsx
+++ b/data/ChaitralisKitchen_ContentPack.xlsx
@@ -832,7 +832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1090,6 +1090,14 @@
 Many vegan and gluten-free options available.</t>
         </is>
       </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Order Sheet Link (Apps Script web app — leave blank to use the Google Form)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2043,7 +2051,6 @@
           <t>Dates (e.g. Oct 1 – Oct 6, 2026)</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2231,8 +2238,6 @@
       <c r="B28" t="n">
         <v>7</v>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>Dry Sabzi</t>
@@ -2248,8 +2253,6 @@
       <c r="B29" t="n">
         <v>8</v>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>Dry Sabzi</t>
@@ -2265,8 +2268,6 @@
       <c r="B30" t="n">
         <v>9</v>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>Dry Sabzi</t>
@@ -2282,8 +2283,6 @@
       <c r="B31" t="n">
         <v>10</v>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>Dry Sabzi</t>
@@ -2299,8 +2298,6 @@
       <c r="B32" t="n">
         <v>11</v>
       </c>
-      <c r="C32" t="inlineStr"/>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>Dry Sabzi</t>
@@ -2316,8 +2313,6 @@
       <c r="B33" t="n">
         <v>12</v>
       </c>
-      <c r="C33" t="inlineStr"/>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>Dry Sabzi</t>

</xml_diff>